<commit_message>
Add spreadsheet audit tooling and fix formula cell protection
</commit_message>
<xml_diff>
--- a/digital-products/excel-source/CashFlowOffice_PaymentScheduler_v1.xlsx
+++ b/digital-products/excel-source/CashFlowOffice_PaymentScheduler_v1.xlsx
@@ -855,7 +855,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="82">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1178,6 +1178,10 @@
     </xf>
     <xf numFmtId="164" fontId="20" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1527,7 +1531,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -1591,7 +1595,7 @@
       <c r="A3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B3" s="81" t="n">
         <f aca="true">TODAY()</f>
         <v>46111</v>
       </c>

</xml_diff>